<commit_message>
Remplace les 8 prospects trop loin de leur ville dans les lots 1 et 2
Les deux premiers lots dataient du rayon de 25 km : un artisan de
Montigny-le-Bretonneux y figurait sous l'etiquette Paris, a 26 km, et
Accueil Auto Pieces 57 sous celle de Metz, a 97 km.

remplace_eloignes.py mesure la distance reelle : il lit l'adresse sur le
site du candidat, resout le code postal aupres de geo.api.gouv.fr et
calcule l'ecart au centre-ville. Un candidat dont la page n'affiche pas
d'adresse n'est pas retenu - c'est cette incertitude qui avait produit le
probleme. Le meme passage ecarte au vol les sites qui parlent de leurs
etablissements au pluriel.

Les 8 remplacants sont a 0,3 a 4,4 km de leur centre-ville, verifies un
par un. Repartition 7 par niche conservee.

Verification finale des deux lots : aucun doublon de domaine, de racine
ni d'enseigne, aucune collision v1, aucune chaine, aucun nom vide,
aucun prospect au-dela de 7 km.
</commit_message>
<xml_diff>
--- a/lot_01.xlsx
+++ b/lot_01.xlsx
@@ -153,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -223,6 +223,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1590,39 +1593,43 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>babacanteen.com</t>
+          <t>resto.krutenau.free.fr</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Baba canteen</t>
+          <t>Winstub La Krutenau</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Toulouse</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr"/>
+          <t>Colmar</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>Colmar (68000)</t>
+        </is>
+      </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I4" s="22" t="inlineStr">
-        <is>
-          <t>oui</t>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr">
@@ -1632,46 +1639,46 @@
       </c>
       <c r="K4" s="12" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (5) | non responsive | document.write | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (3B) | aucun radius/ombre</t>
+          <t>layout en tableaux (23) | &lt;marquee&gt; | bgcolor= | doctype ancien | non responsive | images .gif | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>chezmario.fr</t>
+          <t>babacanteen.com</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Chez Mario</t>
+          <t>Baba canteen</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr"/>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J5" s="20" t="inlineStr">
@@ -1681,46 +1688,46 @@
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>layout en tableaux (4) | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (5) | non responsive | document.write | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (3B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>baan.fr</t>
+          <t>chezmario.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Baan Siam</t>
+          <t>Chez Mario</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr">
-        <is>
-          <t>oui</t>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -1730,46 +1737,46 @@
       </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>layout en tableaux (9) | balises &lt;font&gt; (32) | &lt;center&gt; | bgcolor= | sans doctype | non responsive | images .gif</t>
+          <t>layout en tableaux (4) | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>lechateausormiou.fr</t>
+          <t>baan.fr</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Le Château Sormiou</t>
+          <t>Baan Siam</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="n">
-        <v>47</v>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>57</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J7" s="20" t="inlineStr">
@@ -1779,50 +1786,46 @@
       </c>
       <c r="K7" s="21" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
+          <t>layout en tableaux (9) | balises &lt;font&gt; (32) | &lt;center&gt; | bgcolor= | sans doctype | non responsive | images .gif</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>ldvdraveil.fr</t>
+          <t>lechateausormiou.fr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>La Dolce Vita</t>
+          <t>Le Château Sormiou</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>Draveil (91210)</t>
-        </is>
-      </c>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F8" s="23" t="n">
         <v>47</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
-        <is>
-          <t>oui</t>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -1832,7 +1835,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>layout en tableaux (29) | balises &lt;font&gt; (4) | &lt;center&gt; | non responsive | &lt;br&gt; en masse</t>
+          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
         </is>
       </c>
     </row>
@@ -2553,39 +2556,43 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>cyclolivine.fr</t>
+          <t>atelierdumenager.com</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Cyclolivine</t>
+          <t>Atelier du ménager</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Grenoble</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr"/>
+          <t>Poitiers</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>Poitiers (86000)</t>
+        </is>
+      </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="F5" s="23" t="n">
-        <v>49</v>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>56</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J5" s="20" t="inlineStr">
@@ -2595,46 +2602,46 @@
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>&lt;center&gt; | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (2) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>rustine-beaulieu.weebly.com</t>
+          <t>cyclolivine.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>La Rustine de Beaulieu</t>
+          <t>Cyclolivine</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F6" s="23" t="n">
         <v>49</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="I6" s="22" t="inlineStr">
-        <is>
-          <t>oui</t>
+        <v>8</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -2644,41 +2651,41 @@
       </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>layout en tableaux (4) | balises &lt;font&gt; (29) | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>&lt;center&gt; | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>velosapiens.fr</t>
+          <t>rustine-beaulieu.weebly.com</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Vélo-Sapiens</t>
+          <t>La Rustine de Beaulieu</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F7" s="23" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
+        <v>3</v>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
@@ -2693,60 +2700,56 @@
       </c>
       <c r="K7" s="21" t="inlineStr">
         <is>
-          <t>&lt;center&gt; | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>layout en tableaux (4) | balises &lt;font&gt; (29) | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>laveriedebretagne.free.fr</t>
+          <t>velosapiens.fr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Laverie de Montigny-le-Bretonneux</t>
+          <t>Vélo-Sapiens</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>Montigny-le-Bretonneux (78180)</t>
-        </is>
-      </c>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F8" s="23" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I8" s="22" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>izispot 4.31 (www.izispot.com)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>layout en tableaux (5) | balises &lt;font&gt; (4) | doctype ancien | non responsive</t>
+          <t>&lt;center&gt; | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tolerance de distance portee a 21 km, rayon des villes a 20 km
7 km etait trop severe : une banlieue a 20 km reste demarchable, seuls les
cas aberrants genaient. Six des huit remplacements du commit precedent
sont annules et les prospects d'origine restaures - de 8 a 21 km. Les deux
vrais ecarts sont conserves : Laverie de Montigny (26 km) et Accueil Auto
Pieces 57 (97 km, erreur de placement OSM).

Champ de recherche : 20 km autour des grandes villes, le littoral reste a
7 km car une station balneaire n'a pas de banlieue.

Au passage, delivered.json avait perdu les 60 restaurants de la v1 en
etant reconstruit depuis les seuls lots : ils y sont remis, sans quoi ils
seraient ressortis dans un prochain lot.
</commit_message>
<xml_diff>
--- a/lot_01.xlsx
+++ b/lot_01.xlsx
@@ -1593,43 +1593,39 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>resto.krutenau.free.fr</t>
+          <t>babacanteen.com</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Winstub La Krutenau</t>
+          <t>Baba canteen</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Colmar</t>
-        </is>
-      </c>
-      <c r="D4" s="24" t="inlineStr">
-        <is>
-          <t>Colmar (68000)</t>
-        </is>
-      </c>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr"/>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I4" s="22" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr">
@@ -1639,46 +1635,46 @@
       </c>
       <c r="K4" s="12" t="inlineStr">
         <is>
-          <t>layout en tableaux (23) | &lt;marquee&gt; | bgcolor= | doctype ancien | non responsive | images .gif | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (5) | non responsive | document.write | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (3B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>babacanteen.com</t>
+          <t>chezmario.fr</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Baba canteen</t>
+          <t>Chez Mario</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr"/>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
-        <is>
-          <t>oui</t>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
       <c r="J5" s="20" t="inlineStr">
@@ -1688,46 +1684,46 @@
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (5) | non responsive | document.write | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (3B) | aucun radius/ombre</t>
+          <t>layout en tableaux (4) | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>chezmario.fr</t>
+          <t>baan.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Chez Mario</t>
+          <t>Baan Siam</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -1737,46 +1733,46 @@
       </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>layout en tableaux (4) | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>layout en tableaux (9) | balises &lt;font&gt; (32) | &lt;center&gt; | bgcolor= | sans doctype | non responsive | images .gif</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>baan.fr</t>
+          <t>lechateausormiou.fr</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Baan Siam</t>
+          <t>Le Château Sormiou</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="inlineStr">
         <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="n">
-        <v>57</v>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>47</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
-        <is>
-          <t>oui</t>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
       <c r="J7" s="20" t="inlineStr">
@@ -1786,46 +1782,50 @@
       </c>
       <c r="K7" s="21" t="inlineStr">
         <is>
-          <t>layout en tableaux (9) | balises &lt;font&gt; (32) | &lt;center&gt; | bgcolor= | sans doctype | non responsive | images .gif</t>
+          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>lechateausormiou.fr</t>
+          <t>ldvdraveil.fr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Le Château Sormiou</t>
+          <t>La Dolce Vita</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Marseille</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr"/>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>Draveil (91210)</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F8" s="23" t="n">
         <v>47</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I8" s="22" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
+          <t>layout en tableaux (29) | balises &lt;font&gt; (4) | &lt;center&gt; | non responsive | &lt;br&gt; en masse</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige lot_01 : remplace 19 prospects sur 35 (doublon reel ou visible en resultats organiques)
Verification manuelle via Claude dans Chrome de chaque prospect (recherche de
doublons de site + presence dans les premiers resultats Google organiques
pour "niche + ville") puis remplacement 1:1 par niche, chaque remplacant
re-verifie selon les 2 memes criteres avant acceptation.

Detail : 2 Artisanat/BTP, 3 Beaute, 4 Restauration, 5 Automobile,
5 Services de proximite. Les domaines ecartes (doublons -lpa.fr, associations
benevoles, chaines, societe radiee, site pirate...) sont ajoutes a
delivered.json et aux listes de blacklist pour ne plus jamais ressortir.

Tolerance de distance au centre-ville portee a 22 km (etait 21 km).
</commit_message>
<xml_diff>
--- a/lot_01.xlsx
+++ b/lot_01.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,25 +78,19 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="006B7280"/>
-      <sz val="9"/>
+      <color rgb="00047857"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00047857"/>
-      <sz val="10"/>
+      <color rgb="006B7280"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="0092400E"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00111827"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -153,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -168,7 +162,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,9 +178,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -195,7 +192,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -207,26 +204,17 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -683,12 +671,12 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>multitude-lyon.fr</t>
+          <t>petezki.fr</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Multitude</t>
+          <t>Petezki &amp; Fils</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -703,199 +691,199 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G4" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>macromedia dreamweaver 8</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>layout en tableaux (9) | doctype ancien | non responsive | images .gif | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>ardoise-zinc.fr</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Ardoise et Zinc</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr"/>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G5" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr">
-        <is>
-          <t>layout en tableaux (5) | balises &lt;font&gt; (1) | doctype ancien | non responsive | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>petezki.fr</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Petezki &amp; Fils</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Lyon</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr"/>
-      <c r="E5" s="17" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="n">
-        <v>67</v>
-      </c>
-      <c r="G5" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I5" s="19" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J5" s="20" t="inlineStr">
-        <is>
-          <t>macromedia dreamweaver 8</t>
-        </is>
-      </c>
-      <c r="K5" s="21" t="inlineStr">
-        <is>
-          <t>layout en tableaux (9) | doctype ancien | non responsive | images .gif | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+      <c r="K5" s="22" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (13) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>ardoise-zinc.fr</t>
+          <t>atie-bat.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Ardoise et Zinc</t>
+          <t>Atie Bat</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
         <v>56</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (13) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (2) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>atie-bat.fr</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Atie Bat</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>75</t>
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>biasini-electricite.com</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Biasini</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr"/>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>31</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
         <v>56</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J7" s="20" t="inlineStr">
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K7" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (2) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K7" s="22" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>biasini-electricite.com</t>
+          <t>tech-plomberie.fr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Biasini</t>
+          <t>Tec Plomberie</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Orleans</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F8" s="9" t="n">
@@ -909,117 +897,117 @@
           <t>non</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (3) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>tech-plomberie.fr</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Tec Plomberie</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Orleans</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>45</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>espace-bois-66.com</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Espace Bois Alu PVC</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Perpignan</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr"/>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>66</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="G9" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr">
+        <v>55</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K9" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (3) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="J9" s="21" t="inlineStr">
+        <is>
+          <t>cfirsty®</t>
+        </is>
+      </c>
+      <c r="K9" s="22" t="inlineStr">
+        <is>
+          <t>layout en tableaux (9) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | police vintage</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>verandaconcept.fr</t>
+          <t>fais-ci-fais-ca.com</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Véranda Concept</t>
+          <t>Fais ci Fais ça</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>joomla! - copyright (c) 2005 - 2006 open source matters. all</t>
-        </is>
-      </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>layout en tableaux (7) | doctype ancien | non responsive | pas de @media | pas de flex/grid | aucun radius/ombre</t>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>wordpress 3.0.1</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>&lt;center&gt; | doctype ancien | non responsive | document.write | pas de @media | pas de flex/grid | pas de variables CSS | police vintage</t>
         </is>
       </c>
     </row>
@@ -1168,80 +1156,80 @@
           <t>non</t>
         </is>
       </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr">
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr">
+      <c r="K4" s="13" t="inlineStr">
         <is>
           <t>layout en tableaux (9) | balises &lt;font&gt; (15) | sans doctype | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>ermontbienetre.fr</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Esthétique et Massage de Bien-Être</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>thai-rachawadee.fr</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Thaï Rachawadee</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr"/>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr"/>
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>68</v>
-      </c>
-      <c r="G5" s="17" t="n">
+        <v>66</v>
+      </c>
+      <c r="G5" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I5" s="19" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J5" s="20" t="inlineStr">
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K5" s="21" t="inlineStr">
-        <is>
-          <t>layout en tableaux (8) | bgcolor= | doctype ancien | non responsive | gif de mise en page | images .gif | pas de @media | pas de flex/grid | aucun radius/ombre</t>
+      <c r="K5" s="22" t="inlineStr">
+        <is>
+          <t>bgcolor= | frameset | sans doctype | non responsive | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>thai-rachawadee.fr</t>
+          <t>atelier-arnaud-marie-coiffeur.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Thaï Rachawadee</t>
+          <t>Arnaud Marie</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1256,7 +1244,7 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>6</v>
@@ -1266,95 +1254,95 @@
           <t>non</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
-        <is>
-          <t>bgcolor= | frameset | sans doctype | non responsive | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (4) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>auxonglesdor.free.fr</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Aux Ongles d'Or</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="n">
-        <v>58</v>
-      </c>
-      <c r="G7" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="J7" s="20" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>florentina-linea.fr</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Florentina</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr"/>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>47</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K7" s="21" t="inlineStr">
-        <is>
-          <t>&lt;center&gt; | doctype ancien | non responsive | gif de mise en page | pas de @media | pas de flex/grid | pas de variables CSS | police vintage | aucun radius/ombre</t>
+      <c r="K7" s="22" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>mickaelgreg-coiffure.com</t>
+          <t>institut-beaute-doucebelle.fr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Salon Mixte Barneoud</t>
+          <t>Institut de Beauté Doucebelle</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Annemasse</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="n">
-        <v>58</v>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>46</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>3</v>
@@ -1364,117 +1352,117 @@
           <t>non</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>layout en tableaux (13) | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>atelier-arnaud-marie-coiffeur.fr</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Arnaud Marie</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="G9" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>coiffurestyling.site-solocal.com</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Styling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Nancy</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr"/>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>46</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr">
+      <c r="J9" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K9" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (4) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K9" s="22" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>florentina-linea.fr</t>
+          <t>correiamanuelcoiffeurcreateur.site-solocal.com</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Florentina</t>
+          <t>Mannuel Correia</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>69</t>
         </is>
       </c>
       <c r="F10" s="23" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
@@ -1623,40 +1611,40 @@
           <t>non</t>
         </is>
       </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr">
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr">
+      <c r="K4" s="13" t="inlineStr">
         <is>
           <t>balises &lt;font&gt; (5) | non responsive | document.write | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (3B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>chezmario.fr</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Chez Mario</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr"/>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr"/>
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>33</t>
         </is>
@@ -1664,25 +1652,25 @@
       <c r="F5" s="9" t="n">
         <v>58</v>
       </c>
-      <c r="G5" s="17" t="n">
+      <c r="G5" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="J5" s="20" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K5" s="21" t="inlineStr">
+      <c r="K5" s="22" t="inlineStr">
         <is>
           <t>layout en tableaux (4) | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
@@ -1691,110 +1679,110 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>baan.fr</t>
+          <t>azur-traiteur.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Baan Siam</t>
+          <t>Azur Traiteur</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Aix-en-Provence</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G6" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>joomla! 1.5 - open source content management</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>layout en tableaux (7) | doctype ancien | non responsive | pas de @media | pas de flex/grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>happy-pizz.com</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Happy Pizz - Chez Jo</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Quimper</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr"/>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>49</v>
+      </c>
+      <c r="G7" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
-        <is>
-          <t>layout en tableaux (9) | balises &lt;font&gt; (32) | &lt;center&gt; | bgcolor= | sans doctype | non responsive | images .gif</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>lechateausormiou.fr</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Le Château Sormiou</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Marseille</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="n">
-        <v>47</v>
-      </c>
-      <c r="G7" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="J7" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K7" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
+      <c r="K7" s="22" t="inlineStr">
+        <is>
+          <t>bgcolor= | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>ldvdraveil.fr</t>
+          <t>boucherie-economique.fr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>La Dolce Vita</t>
+          <t>La boucherie économique</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1802,138 +1790,134 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>Draveil (91210)</t>
-        </is>
-      </c>
+      <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
       <c r="F8" s="23" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>layout en tableaux (29) | balises &lt;font&gt; (4) | &lt;center&gt; | non responsive | &lt;br&gt; en masse</t>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>chapitre6.fr</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Chapitre VI</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Lille</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>59</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>coignacsarl.site-solocal.com</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Maison Coignac</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Limoges</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr"/>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>87</t>
         </is>
       </c>
       <c r="F9" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="G9" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="J9" s="20" t="inlineStr">
+        <v>46</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K9" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (1) | bgcolor= | frameset | sans doctype | non responsive</t>
+      <c r="K9" s="22" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>laovientiane.fr</t>
+          <t>chapitre6.fr</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Lao Vientiane</t>
+          <t>Chapitre VI</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>59</t>
         </is>
       </c>
       <c r="F10" s="23" t="n">
         <v>45</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>&lt;center&gt; | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (1) | bgcolor= | frameset | sans doctype | non responsive</t>
         </is>
       </c>
     </row>
@@ -2087,308 +2071,308 @@
           <t>non</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr">
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr">
+      <c r="K4" s="13" t="inlineStr">
         <is>
           <t>layout en tableaux (5) | balises &lt;font&gt; (1) | doctype ancien | non responsive | gif de mise en page | images .gif | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>garage-laban-rouen.fr</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Garage Laban</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Rouen</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr"/>
-      <c r="E5" s="17" t="inlineStr">
-        <is>
-          <t>76</t>
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>belr-automobiles.com</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Bel'R Automobiles</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>La Rochelle</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr"/>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>17</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="G5" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G5" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I5" s="19" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J5" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K5" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (16) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="J5" s="21" t="inlineStr">
+        <is>
+          <t>lmsoft web creator pro, version:6.0.0.4</t>
+        </is>
+      </c>
+      <c r="K5" s="22" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (29) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>autopieces35.fr</t>
+          <t>autopremium-66.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Auto Pièces 35</t>
+          <t>Top Garage Auto Premium 66</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Perpignan</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>56</v>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>46</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (10) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>carrosserie-adamo.com</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Carrosserie Adamo</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>garage-des-mines.fr</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Garage des Mines</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Saint-Etienne</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr"/>
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>42</t>
         </is>
       </c>
-      <c r="F7" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="G7" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="F7" s="23" t="n">
+        <v>46</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J7" s="20" t="inlineStr">
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K7" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (31) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K7" s="22" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>carrosserie-barcelona.fr</t>
+          <t>garageabauto.site-solocal.com</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Carrosserie Barcelona</t>
+          <t>AB Auto</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Bayonne</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>64</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="n">
-        <v>56</v>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>46</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (5) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>carrosserievernoise.fr</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Carrosserie Vernoise</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Rennes</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="G9" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>garagedelapaix.site-solocal.com</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Garage de la Paix</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr"/>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>46</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr">
+      <c r="J9" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K9" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (7) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K9" s="22" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>belr-automobiles.com</t>
+          <t>ad69.fr</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Bel'R Automobiles</t>
+          <t>AutoDiscount 69</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>La Rochelle</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="n">
-        <v>50</v>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>42</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>lmsoft web creator pro, version:6.0.0.4</t>
-        </is>
-      </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (29) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>webdev</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>layout en tableaux (193) | non responsive | document.write | pas de flex/grid | police vintage</t>
         </is>
       </c>
     </row>
@@ -2507,12 +2491,12 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>velocipaide.fr</t>
+          <t>sapah.fr</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Vélocipaide</t>
+          <t>Sapah</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -2527,82 +2511,78 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>dreamweaver cs4, photoshop cs4, firework cs4</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>doctype ancien | non responsive | gif de mise en page | images .gif | document.write | pas de @media | pas de flex/grid | pas de variables CSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>abaqueinformatique.com</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>@baque Informatique</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>La Rochelle</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr"/>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="G5" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr">
-        <is>
-          <t>bueno 1.5.1</t>
-        </is>
-      </c>
-      <c r="K4" s="12" t="inlineStr">
-        <is>
-          <t>&lt;center&gt; | bgcolor= | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (2B) | aucun radius/ombre</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>atelierdumenager.com</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Atelier du ménager</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Poitiers</t>
-        </is>
-      </c>
-      <c r="D5" s="25" t="inlineStr">
-        <is>
-          <t>Poitiers (86000)</t>
-        </is>
-      </c>
-      <c r="E5" s="17" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="G5" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I5" s="19" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J5" s="20" t="inlineStr">
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K5" s="21" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (2) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+      <c r="K5" s="22" t="inlineStr">
+        <is>
+          <t>doctype ancien | non responsive | images .gif | pas de @media | pas de flex/grid | pas de variables CSS | police vintage | aucun radius/ombre</t>
         </is>
       </c>
     </row>
@@ -2644,173 +2624,173 @@
           <t>non</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
+      <c r="K6" s="13" t="inlineStr">
         <is>
           <t>&lt;center&gt; | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>rustine-beaulieu.weebly.com</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>La Rustine de Beaulieu</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Rennes</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>35</t>
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>coeur-de-poil.fr</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Cœur de Poil</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Nancy</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr"/>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>54</t>
         </is>
       </c>
       <c r="F7" s="23" t="n">
-        <v>49</v>
-      </c>
-      <c r="G7" s="17" t="n">
+        <v>46</v>
+      </c>
+      <c r="G7" s="18" t="n">
         <v>3</v>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J7" s="20" t="inlineStr">
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K7" s="21" t="inlineStr">
-        <is>
-          <t>layout en tableaux (4) | balises &lt;font&gt; (29) | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+      <c r="K7" s="22" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>velosapiens.fr</t>
+          <t>label-image-78.com</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Vélo-Sapiens</t>
+          <t>Label Im@ge 78</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F8" s="23" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>&lt;center&gt; | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>jpcycles.sitego.fr</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>JP Cycles</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>75</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>lypart-studio.com</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Lypa'rt Studio</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Le Mans</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr"/>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>72</t>
         </is>
       </c>
       <c r="F9" s="23" t="n">
-        <v>37</v>
-      </c>
-      <c r="G9" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="G9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K9" s="21" t="inlineStr">
-        <is>
-          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
+      <c r="J9" s="21" t="inlineStr">
+        <is>
+          <t>webacappella 4.6.27  professional (osx) #22c4</t>
+        </is>
+      </c>
+      <c r="K9" s="22" t="inlineStr">
+        <is>
+          <t>doctype ancien | non responsive | document.write | pas de @media | pas de flex/grid</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>archphoenix.team</t>
+          <t>jpcycles.sitego.fr</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>ArchPhénix Team (Atelier de Paris)</t>
+          <t>JP Cycles</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -2825,29 +2805,29 @@
         </is>
       </c>
       <c r="F10" s="23" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="22" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>layout en tableaux (3) | pas de @media | pas de flex/grid | aucun radius/ombre</t>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verifie systematiquement la distance des 19 remplacants du lot_01 et corrige un bug de desambiguisation de code postal
coord_cp() prenait le premier resultat de l'API geo pour un code postal,
alors qu'un meme code postal peut couvrir plusieurs communes (87400 =
Saint-Leonard-de-Noblat OU Champnetery ; 66600 = Rivesaltes OU Calce). Le
nom de la commune, deja lu sur la page du prospect, est maintenant utilise
pour choisir la bonne parmi les resultats retournes.

Toutes les distances des 19 remplacants sont desormais dans la colonne
commune et confirmees < 22 km (le plus loin : Toul -> Nancy, 21.1 km).
Lots 2 a 4 rejoues avec le script corrige : aucun probleme detecte, mais
la colonne commune n'y est renseignee que pour 6 a 7 lignes sur 35 - la
grande majorite des prospects de ces lots n'ont jamais ete verifies par
ce script et reposent uniquement sur l'etiquette ville d'origine.
</commit_message>
<xml_diff>
--- a/lot_01.xlsx
+++ b/lot_01.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,6 +85,12 @@
       <name val="Calibri"/>
       <color rgb="006B7280"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00111827"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -147,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -213,8 +219,14 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -929,7 +941,11 @@
           <t>Perpignan</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr"/>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Saint-Laurent-de-la-Salanque (66250)</t>
+        </is>
+      </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
           <t>66</t>
@@ -1292,7 +1308,7 @@
           <t>44</t>
         </is>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="24" t="n">
         <v>47</v>
       </c>
       <c r="G7" s="18" t="n">
@@ -1341,7 +1357,7 @@
           <t>74</t>
         </is>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G8" s="8" t="n">
@@ -1384,13 +1400,17 @@
           <t>Nancy</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr"/>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Frouard (54390)</t>
+        </is>
+      </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G9" s="18" t="n">
@@ -1433,13 +1453,17 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr"/>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>Pusignan (69330)</t>
+        </is>
+      </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
           <t>69</t>
         </is>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G10" s="8" t="n">
@@ -1747,7 +1771,7 @@
           <t>29</t>
         </is>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="24" t="n">
         <v>49</v>
       </c>
       <c r="G7" s="18" t="n">
@@ -1790,13 +1814,17 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr"/>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>Versailles (78000)</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G8" s="8" t="n">
@@ -1839,13 +1867,17 @@
           <t>Limoges</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr"/>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Saint-Leonard-de-Noblat (87400)</t>
+        </is>
+      </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
           <t>87</t>
         </is>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G9" s="18" t="n">
@@ -1894,7 +1926,7 @@
           <t>59</t>
         </is>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>45</v>
       </c>
       <c r="G10" s="8" t="n">
@@ -2147,13 +2179,17 @@
           <t>Perpignan</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr"/>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>Rivesaltes (66600)</t>
+        </is>
+      </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
           <t>66</t>
         </is>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G6" s="8" t="n">
@@ -2196,13 +2232,17 @@
           <t>Saint-Etienne</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr"/>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>La Ricamarie (42150)</t>
+        </is>
+      </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
           <t>42</t>
         </is>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G7" s="18" t="n">
@@ -2245,13 +2285,17 @@
           <t>Nancy</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr"/>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>Toul (54200)</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G8" s="8" t="n">
@@ -2294,13 +2338,17 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr"/>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Le Perreux-sur-Marne (94170)</t>
+        </is>
+      </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G9" s="18" t="n">
@@ -2343,13 +2391,17 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr"/>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>Saint-Bonnet-de-Mure (69720)</t>
+        </is>
+      </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
           <t>69</t>
         </is>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>42</v>
       </c>
       <c r="G10" s="8" t="n">
@@ -2504,7 +2556,11 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr"/>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>Villeneuve-Saint-Georges (94190)</t>
+        </is>
+      </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
           <t>75</t>
@@ -2553,7 +2609,11 @@
           <t>La Rochelle</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr"/>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>L'Houmeau (17137)</t>
+        </is>
+      </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
           <t>17</t>
@@ -2608,7 +2668,7 @@
           <t>38</t>
         </is>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="24" t="n">
         <v>49</v>
       </c>
       <c r="G6" s="8" t="n">
@@ -2651,13 +2711,17 @@
           <t>Nancy</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr"/>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>Champigneulles (54250)</t>
+        </is>
+      </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="24" t="n">
         <v>46</v>
       </c>
       <c r="G7" s="18" t="n">
@@ -2700,13 +2764,17 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr"/>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>Houilles (78800)</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="24" t="n">
         <v>44</v>
       </c>
       <c r="G8" s="8" t="n">
@@ -2755,7 +2823,7 @@
           <t>72</t>
         </is>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="24" t="n">
         <v>42</v>
       </c>
       <c r="G9" s="18" t="n">
@@ -2804,7 +2872,7 @@
           <t>75</t>
         </is>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>37</v>
       </c>
       <c r="G10" s="8" t="n">

</xml_diff>

<commit_message>
Verifie les 35 prospects du lot_01 pour fermeture definitive, remplace 3 enseignes
Chaque enseigne du lot_01 verifiee sur Google Maps (statut "Definitivement
ferme" ou non). 2 fermetures confirmees :
- chezmario.fr (Chez Mario, Bordeaux) -- devenu "Aux deux saveurs"
- chapitre6.fr (Chapitre VI, Templeuve-en-Pevele)

Une 3e enseigne retiree pour un motif different decouvert au passage :
atie-bat.fr a en realite 3 adresses actives a Paris sous la meme enseigne
(chaine non detectee lors des verifications precedentes).

Remplacants verifies selon le meme protocole (doublon + resultats
organiques Google) et ouverture confirmee sur Maps.

Ecarte aussi au passage : une boulangerie en chaine dont 2 des 4 enseignes
sont deja "Definitivement fermees", un cafe associatif, et un ostreiculteur
sous la menace d'une liquidation judiciaire (presse locale).
</commit_message>
<xml_diff>
--- a/lot_01.xlsx
+++ b/lot_01.xlsx
@@ -219,13 +219,13 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -781,23 +781,23 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>atie-bat.fr</t>
+          <t>biasini-electricite.com</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Atie Bat</t>
+          <t>Biasini</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
@@ -823,30 +823,30 @@
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (2) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>biasini-electricite.com</t>
+          <t>tech-plomberie.fr</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Biasini</t>
+          <t>Tec Plomberie</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Orleans</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr"/>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
@@ -872,37 +872,41 @@
       </c>
       <c r="K7" s="22" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (3) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>tech-plomberie.fr</t>
+          <t>espace-bois-66.com</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Tec Plomberie</t>
+          <t>Espace Bois Alu PVC</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Orleans</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr"/>
+          <t>Perpignan</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Saint-Laurent-de-la-Salanque (66250)</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>66</t>
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
@@ -916,46 +920,42 @@
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>cfirsty®</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (3) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>layout en tableaux (9) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | police vintage</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>espace-bois-66.com</t>
+          <t>fais-ci-fais-ca.com</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Espace Bois Alu PVC</t>
+          <t>Fais ci Fais ça</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Perpignan</t>
-        </is>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>Saint-Laurent-de-la-Salanque (66250)</t>
-        </is>
-      </c>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr"/>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G9" s="18" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
@@ -969,42 +969,46 @@
       </c>
       <c r="J9" s="21" t="inlineStr">
         <is>
-          <t>cfirsty®</t>
+          <t>wordpress 3.0.1</t>
         </is>
       </c>
       <c r="K9" s="22" t="inlineStr">
         <is>
-          <t>layout en tableaux (9) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | police vintage</t>
+          <t>&lt;center&gt; | doctype ancien | non responsive | document.write | pas de @media | pas de flex/grid | pas de variables CSS | police vintage</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>fais-ci-fais-ca.com</t>
+          <t>lorconcept-toiture.com</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Fais ci Fais ça</t>
+          <t>Lor'Concept Toiture</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr"/>
+          <t>Nancy</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>Tomblaine (54510)</t>
+        </is>
+      </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="n">
-        <v>54</v>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>38</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
@@ -1018,12 +1022,12 @@
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>wordpress 3.0.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>&lt;center&gt; | doctype ancien | non responsive | document.write | pas de @media | pas de flex/grid | pas de variables CSS | police vintage</t>
+          <t>doctype ancien | non responsive | pas de @media | pas de flex/grid</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1404,7 @@
           <t>Nancy</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>Frouard (54390)</t>
         </is>
@@ -1453,7 +1457,7 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>Pusignan (69330)</t>
         </is>
@@ -1654,79 +1658,79 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>chezmario.fr</t>
+          <t>azur-traiteur.fr</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Chez Mario</t>
+          <t>Azur Traiteur</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Aix-en-Provence</t>
         </is>
       </c>
       <c r="D5" s="17" t="inlineStr"/>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="G5" s="18" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J5" s="21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>joomla! 1.5 - open source content management</t>
         </is>
       </c>
       <c r="K5" s="22" t="inlineStr">
         <is>
-          <t>layout en tableaux (4) | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>layout en tableaux (7) | doctype ancien | non responsive | pas de @media | pas de flex/grid</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>azur-traiteur.fr</t>
+          <t>happy-pizz.com</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Azur Traiteur</t>
+          <t>Happy Pizz - Chez Jo</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Aix-en-Provence</t>
+          <t>Quimper</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>52</v>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>49</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
@@ -1740,42 +1744,46 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>joomla! 1.5 - open source content management</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>layout en tableaux (7) | doctype ancien | non responsive | pas de @media | pas de flex/grid</t>
+          <t>bgcolor= | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>happy-pizz.com</t>
+          <t>boucherie-economique.fr</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Happy Pizz - Chez Jo</t>
+          <t>La boucherie économique</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Quimper</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr"/>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>Versailles (78000)</t>
+        </is>
+      </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F7" s="24" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
@@ -1794,34 +1802,34 @@
       </c>
       <c r="K7" s="22" t="inlineStr">
         <is>
-          <t>bgcolor= | doctype ancien | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>boucherie-economique.fr</t>
+          <t>coignacsarl.site-solocal.com</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>La boucherie économique</t>
+          <t>Maison Coignac</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D8" s="25" t="inlineStr">
-        <is>
-          <t>Versailles (78000)</t>
+          <t>Limoges</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Saint-Leonard-de-Noblat (87400)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>87</t>
         </is>
       </c>
       <c r="F8" s="24" t="n">
@@ -1854,34 +1862,34 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>coignacsarl.site-solocal.com</t>
+          <t>cafedesarts.alwaysdata.net</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Maison Coignac</t>
+          <t>Café des Arts</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Limoges</t>
-        </is>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>Saint-Leonard-de-Noblat (87400)</t>
+          <t>Caen</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>Herouville-Saint-Clair (14200)</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G9" s="18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
@@ -1900,46 +1908,46 @@
       </c>
       <c r="K9" s="22" t="inlineStr">
         <is>
-          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>&lt;center&gt; | non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>chapitre6.fr</t>
+          <t>restaurant-ariana.com</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Chapitre VI</t>
+          <t>L'Ariana</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>44</t>
         </is>
       </c>
       <c r="F10" s="24" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
@@ -1949,7 +1957,7 @@
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (1) | bgcolor= | frameset | sans doctype | non responsive</t>
+          <t>balises &lt;font&gt; (1) | non responsive | pas de @media</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2187,7 @@
           <t>Perpignan</t>
         </is>
       </c>
-      <c r="D6" s="25" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>Rivesaltes (66600)</t>
         </is>
@@ -2232,7 +2240,7 @@
           <t>Saint-Etienne</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="25" t="inlineStr">
         <is>
           <t>La Ricamarie (42150)</t>
         </is>
@@ -2285,7 +2293,7 @@
           <t>Nancy</t>
         </is>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Toul (54200)</t>
         </is>
@@ -2338,7 +2346,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>Le Perreux-sur-Marne (94170)</t>
         </is>
@@ -2391,7 +2399,7 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>Saint-Bonnet-de-Mure (69720)</t>
         </is>
@@ -2556,7 +2564,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="23" t="inlineStr">
         <is>
           <t>Villeneuve-Saint-Georges (94190)</t>
         </is>
@@ -2609,7 +2617,7 @@
           <t>La Rochelle</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>L'Houmeau (17137)</t>
         </is>
@@ -2711,7 +2719,7 @@
           <t>Nancy</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="25" t="inlineStr">
         <is>
           <t>Champigneulles (54250)</t>
         </is>
@@ -2764,7 +2772,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Houilles (78800)</t>
         </is>

</xml_diff>